<commit_message>
Weekly refresh of the Livingry Dashboard extracts
</commit_message>
<xml_diff>
--- a/reports/livingry_dashboard.xlsx
+++ b/reports/livingry_dashboard.xlsx
@@ -913,7 +913,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>United States GDP per capita (constant 2015 dollars): $39,200 in 1990, $67,946 in 2025. Mauna Loa annual mean, full years only: 354.5 ppm in 1990, 427.3 ppm in 2025. Latest month: 427.55 ppm in 2026-08.</t>
+          <t>United States GDP per capita (constant 2015 dollars): $39,200 in 1990, $67,946 in 2025. Mauna Loa annual mean, full years only: 354.5 ppm in 1990, 427.3 ppm in 2025. Latest month: 426.07 ppm in 2026-09.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -3257,7 +3257,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>427.55</t>
+          <t>426.07</t>
         </is>
       </c>
     </row>

</xml_diff>